<commit_message>
work on OC and price_limit bags
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0708A4E6-49BE-4C40-A9E4-908FC9D529E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79947B38-ADA6-402B-BFF0-903C6756C414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="466">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1457,6 +1457,12 @@
   </si>
   <si>
     <t>Анализ, фикс проблем</t>
+  </si>
+  <si>
+    <t>Работа над OrderCords</t>
+  </si>
+  <si>
+    <t>Убрал систему large</t>
   </si>
 </sst>
 </file>
@@ -5204,6 +5210,12 @@
       <c r="E4" t="s">
         <v>31</v>
       </c>
+      <c r="F4" s="3">
+        <v>46283</v>
+      </c>
+      <c r="G4" t="s">
+        <v>465</v>
+      </c>
       <c r="H4" t="s">
         <v>37</v>
       </c>
@@ -12253,6 +12265,12 @@
       <c r="B2" t="s">
         <v>28</v>
       </c>
+      <c r="C2" s="3">
+        <v>46283</v>
+      </c>
+      <c r="D2" t="s">
+        <v>464</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">

</xml_diff>

<commit_message>
try new zigzag again
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5607667F-174C-434C-83ED-4E4553462BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A3556B-33B2-46C3-8ACA-7A6ACED81749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,6 +21,7 @@
     <sheet name="ТекПроблем" sheetId="6" r:id="rId6"/>
     <sheet name="Анализ нейронки стратегий" sheetId="7" r:id="rId7"/>
     <sheet name="Работа" sheetId="8" r:id="rId8"/>
+    <sheet name="Текущие задачи" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="483">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1478,6 +1479,42 @@
   </si>
   <si>
     <t>add_zigzag_window_210926</t>
+  </si>
+  <si>
+    <t>Работал над зигзагом 220926</t>
+  </si>
+  <si>
+    <t>Ордер тест</t>
+  </si>
+  <si>
+    <t>Получение ленты</t>
+  </si>
+  <si>
+    <t>Получение кластеров</t>
+  </si>
+  <si>
+    <t>Зигзаг</t>
+  </si>
+  <si>
+    <t>Починка алгоритмов</t>
+  </si>
+  <si>
+    <t>Улучшение алгоритмов</t>
+  </si>
+  <si>
+    <t>Создание новых VEG</t>
+  </si>
+  <si>
+    <t>Создание новых WEG</t>
+  </si>
+  <si>
+    <t>Создание ST1</t>
+  </si>
+  <si>
+    <t>Создание робота на зебре</t>
+  </si>
+  <si>
+    <t>Создание SEGML c обучением на истории</t>
   </si>
 </sst>
 </file>
@@ -12309,7 +12346,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD57C989-6F2B-410E-8934-538033C06A98}">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
@@ -12402,6 +12439,12 @@
       <c r="B10" t="s">
         <v>440</v>
       </c>
+      <c r="C10" s="3">
+        <v>46287</v>
+      </c>
+      <c r="D10" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
@@ -12413,31 +12456,2052 @@
       <c r="Q12" s="12"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
       <c r="Q13" s="12"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
       <c r="Q14" s="12"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
       <c r="Q15" s="12"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
       <c r="Q16" s="12"/>
     </row>
-    <row r="17" spans="17:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>48</v>
+      </c>
       <c r="Q17" s="12"/>
     </row>
-    <row r="18" spans="17:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>48</v>
+      </c>
       <c r="Q18" s="12"/>
     </row>
-    <row r="19" spans="17:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>50</v>
+      </c>
       <c r="Q19" s="12"/>
     </row>
-    <row r="20" spans="17:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
       <c r="Q20" s="12"/>
+    </row>
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>440</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10B68135-0511-4A43-8FE7-1FF0E8B64F45}">
+  <dimension ref="A2:G378"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="7" width="39.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C3" t="s">
+        <v>476</v>
+      </c>
+      <c r="D3" t="s">
+        <v>476</v>
+      </c>
+      <c r="E3" t="s">
+        <v>477</v>
+      </c>
+      <c r="F3" t="s">
+        <v>476</v>
+      </c>
+      <c r="G3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>473</v>
+      </c>
+      <c r="C4" t="s">
+        <v>477</v>
+      </c>
+      <c r="D4" t="s">
+        <v>477</v>
+      </c>
+      <c r="E4" t="s">
+        <v>478</v>
+      </c>
+      <c r="F4" t="s">
+        <v>477</v>
+      </c>
+      <c r="G4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>474</v>
+      </c>
+      <c r="E5" t="s">
+        <v>479</v>
+      </c>
+      <c r="G5" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>475</v>
+      </c>
+      <c r="G6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A315">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A316">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A317">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A318">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A319">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A320">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A321">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A322">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A323">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A324">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A325">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A326">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A327">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A328">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A329">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A330">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A331">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A332">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A333">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A334">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A335">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A336">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A337">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A338">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A339">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A340">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A341">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A342">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A345">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A346">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A347">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A348">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A350">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A351">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A352">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A353">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A354">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A357">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A358">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A359">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A360">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A361">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A362">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A363">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A364">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A365">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A366">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A367">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A368">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A369">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A370">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A371">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A372">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A373">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A374">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A378">
+        <v>376</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add new ws UEG7 on add_average_fractals_window
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF58C30-0039-4BD1-B24A-8EA696AB6AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D38D178-48F9-4C1C-BCB5-6F9856B20876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="494">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1523,9 +1523,6 @@
     <t>UEG8_SOLDIER</t>
   </si>
   <si>
-    <t>AVENGER на add_zigzag_window_210926</t>
-  </si>
-  <si>
     <t>Новая версия на add_zigzag_window_210926</t>
   </si>
   <si>
@@ -1538,10 +1535,19 @@
     <t>Разработка UEG8</t>
   </si>
   <si>
-    <t>UEG8_DETECTIVE</t>
-  </si>
-  <si>
-    <t>Soldier с дополнительными настройками</t>
+    <t>AVENGER на add_zigzag_window_210926 с доп настройками</t>
+  </si>
+  <si>
+    <t>UEG7_LOVERGOOSE</t>
+  </si>
+  <si>
+    <t>UEG7_DODO на add_average_fractals_window</t>
+  </si>
+  <si>
+    <t>UEG7_LOVERDUCK</t>
+  </si>
+  <si>
+    <t>UEG7_DUELDODO на add_average_fractals_window</t>
   </si>
 </sst>
 </file>
@@ -5258,7 +5264,7 @@
       </c>
       <c r="O2">
         <f>COUNTIF(D:D,O1)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P2">
         <f>COUNTIF(D:D,P1)</f>
@@ -7256,7 +7262,7 @@
         <v>50</v>
       </c>
       <c r="E114" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
@@ -7264,7 +7270,7 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C115" s="3">
         <v>46290</v>
@@ -7273,7 +7279,7 @@
         <v>48</v>
       </c>
       <c r="E115" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -7296,6 +7302,18 @@
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>492</v>
+      </c>
+      <c r="C117" s="3">
+        <v>46290</v>
+      </c>
+      <c r="D117" t="s">
+        <v>50</v>
+      </c>
+      <c r="E117" t="s">
+        <v>493</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
@@ -12466,7 +12484,7 @@
         <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -12477,7 +12495,7 @@
         <v>46290</v>
       </c>
       <c r="D6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
some work again again
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA36891B-FEB0-43B4-96CB-9E74B1DC5A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D49512-D9F8-40A0-A622-45DEDC9CDBB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="519">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="523">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1623,6 +1623,18 @@
   </si>
   <si>
     <t>Добавление step action</t>
+  </si>
+  <si>
+    <t>Анализ оптимизации, результатов</t>
+  </si>
+  <si>
+    <t>PEG30_ETC2</t>
+  </si>
+  <si>
+    <t>Робот с заявками на шаг от close со спредом</t>
+  </si>
+  <si>
+    <t>Работа со spred action</t>
   </si>
 </sst>
 </file>
@@ -1748,10 +1760,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -2085,7 +2097,7 @@
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -2093,13 +2105,13 @@
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="16"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2107,43 +2119,43 @@
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="16"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="16"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="16"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="16"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="16"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
@@ -5334,7 +5346,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(D:D,L1)</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M2">
         <f>COUNTIF(D:D,M1)</f>
@@ -5551,7 +5563,7 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>53</v>
       </c>
       <c r="C13" s="3">
@@ -5705,7 +5717,7 @@
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>310</v>
       </c>
       <c r="C21" s="3">
@@ -5722,7 +5734,7 @@
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>311</v>
       </c>
       <c r="C22" s="3">
@@ -5739,7 +5751,7 @@
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="16" t="s">
         <v>312</v>
       </c>
       <c r="C23" s="3">
@@ -5756,7 +5768,7 @@
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="16" t="s">
         <v>313</v>
       </c>
       <c r="C24" s="3">
@@ -5790,7 +5802,7 @@
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="16" t="s">
         <v>315</v>
       </c>
       <c r="C26" s="3">
@@ -5841,7 +5853,7 @@
       <c r="A29">
         <v>28</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="16" t="s">
         <v>318</v>
       </c>
       <c r="C29" s="3">
@@ -6371,7 +6383,7 @@
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="16" t="s">
         <v>346</v>
       </c>
       <c r="C57" s="3">
@@ -6405,7 +6417,7 @@
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59" s="17" t="s">
+      <c r="B59" s="16" t="s">
         <v>348</v>
       </c>
       <c r="C59" s="3">
@@ -6422,7 +6434,7 @@
       <c r="A60">
         <v>59</v>
       </c>
-      <c r="B60" s="17" t="s">
+      <c r="B60" s="16" t="s">
         <v>349</v>
       </c>
       <c r="C60" s="3">
@@ -6439,7 +6451,7 @@
       <c r="A61">
         <v>60</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="16" t="s">
         <v>350</v>
       </c>
       <c r="C61" s="3">
@@ -6524,7 +6536,7 @@
       <c r="A66">
         <v>65</v>
       </c>
-      <c r="B66" s="17" t="s">
+      <c r="B66" s="16" t="s">
         <v>355</v>
       </c>
       <c r="C66" s="3">
@@ -6541,7 +6553,7 @@
       <c r="A67">
         <v>66</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="16" t="s">
         <v>356</v>
       </c>
       <c r="C67" s="3">
@@ -7239,7 +7251,7 @@
       <c r="A107">
         <v>106</v>
       </c>
-      <c r="B107" s="17" t="s">
+      <c r="B107" s="16" t="s">
         <v>447</v>
       </c>
       <c r="C107" s="3">
@@ -7341,7 +7353,7 @@
       <c r="A113">
         <v>112</v>
       </c>
-      <c r="B113" s="17" t="s">
+      <c r="B113" s="16" t="s">
         <v>465</v>
       </c>
       <c r="C113" s="3">
@@ -7426,7 +7438,7 @@
       <c r="A118">
         <v>117</v>
       </c>
-      <c r="B118" s="17" t="s">
+      <c r="B118" s="16" t="s">
         <v>491</v>
       </c>
       <c r="C118" s="3">
@@ -7443,7 +7455,7 @@
       <c r="A119">
         <v>118</v>
       </c>
-      <c r="B119" s="17" t="s">
+      <c r="B119" s="16" t="s">
         <v>493</v>
       </c>
       <c r="C119" s="3">
@@ -7528,7 +7540,7 @@
       <c r="A124">
         <v>123</v>
       </c>
-      <c r="B124" s="17" t="s">
+      <c r="B124" s="16" t="s">
         <v>498</v>
       </c>
       <c r="C124" s="3">
@@ -7595,6 +7607,18 @@
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>520</v>
+      </c>
+      <c r="C128" s="3">
+        <v>46297</v>
+      </c>
+      <c r="D128" t="s">
+        <v>12</v>
+      </c>
+      <c r="E128" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
@@ -12705,7 +12729,7 @@
       </c>
       <c r="F2">
         <f>COUNTIF(B:B,F1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2">
         <f>COUNTIF(B:B,G1)</f>
@@ -12729,7 +12753,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(B:B,L1)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -12878,11 +12902,29 @@
       <c r="A13">
         <v>12</v>
       </c>
+      <c r="B13" t="s">
+        <v>506</v>
+      </c>
+      <c r="C13" s="3">
+        <v>46295</v>
+      </c>
+      <c r="D13" t="s">
+        <v>519</v>
+      </c>
       <c r="Q13" s="12"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="3">
+        <v>46297</v>
+      </c>
+      <c r="D14" t="s">
+        <v>522</v>
       </c>
       <c r="Q14" s="12"/>
     </row>

</xml_diff>

<commit_message>
add some indicators and record 216 rubles
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B18D9D-B75E-40F5-AE1A-8E145BCFED69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE92AF34-E7AD-49A6-A56E-8307045083E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="628">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1902,9 +1902,6 @@
     <t>percentle rank</t>
   </si>
   <si>
-    <t>blendaer score</t>
-  </si>
-  <si>
     <t>Робот дебатер</t>
   </si>
   <si>
@@ -1942,6 +1939,18 @@
   </si>
   <si>
     <t>Канал по макс и мин отношению (отклонению?)</t>
+  </si>
+  <si>
+    <t>Индикатор моментум</t>
+  </si>
+  <si>
+    <t>Индикатор Монте-Карло</t>
+  </si>
+  <si>
+    <t>Посмотреть индикаторы на TV, которых у нас нет</t>
+  </si>
+  <si>
+    <t>blender score</t>
   </si>
 </sst>
 </file>
@@ -2392,19 +2401,20 @@
   <dimension ref="A1:C368"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="84.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>605</v>
       </c>
       <c r="C2">
@@ -2415,7 +2425,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>606</v>
       </c>
       <c r="C3">
@@ -2426,7 +2436,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>607</v>
       </c>
       <c r="C4">
@@ -2437,7 +2447,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>608</v>
       </c>
       <c r="C5">
@@ -2448,7 +2458,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>609</v>
       </c>
       <c r="C6">
@@ -2459,7 +2469,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>610</v>
       </c>
       <c r="C7">
@@ -2470,8 +2480,8 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>611</v>
+      <c r="B8" s="4" t="s">
+        <v>627</v>
       </c>
       <c r="C8">
         <v>3</v>
@@ -2481,8 +2491,8 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>617</v>
+      <c r="B9" s="4" t="s">
+        <v>616</v>
       </c>
       <c r="C9">
         <v>3</v>
@@ -2493,7 +2503,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -2504,7 +2514,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C11">
         <v>3</v>
@@ -2581,7 +2591,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -2647,7 +2657,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -2658,7 +2668,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -2669,10 +2679,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>594</v>
+        <v>626</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2680,7 +2690,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>567</v>
+        <v>594</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -2691,7 +2701,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -2702,7 +2712,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -2713,7 +2723,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -2724,7 +2734,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -2735,7 +2745,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -2746,7 +2756,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -2757,7 +2767,7 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -2768,7 +2778,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -2779,7 +2789,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -2790,7 +2800,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -2801,7 +2811,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -2812,7 +2822,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -2823,7 +2833,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -2834,7 +2844,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2845,7 +2855,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -2856,7 +2866,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2867,7 +2877,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -2878,7 +2888,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2889,7 +2899,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>624</v>
+        <v>590</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2900,7 +2910,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>591</v>
+        <v>623</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -2911,7 +2921,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -2922,7 +2932,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -2933,7 +2943,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -2944,7 +2954,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2955,7 +2965,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2966,7 +2976,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -2977,7 +2987,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -2988,7 +2998,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>614</v>
+        <v>603</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -2999,7 +3009,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -3010,7 +3020,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -3021,7 +3031,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -3032,7 +3042,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -3042,16 +3052,34 @@
       <c r="A60">
         <v>59</v>
       </c>
+      <c r="B60" t="s">
+        <v>620</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
+      <c r="B61" t="s">
+        <v>624</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
+      <c r="B62" t="s">
+        <v>625</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63">
@@ -4584,8 +4612,8 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C369">
-    <sortCondition descending="1" ref="C2:C369"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C368">
+    <sortCondition descending="1" ref="C2:C368"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add new bots peg17 and peg26
</commit_message>
<xml_diff>
--- a/__docs/RoadMap.xlsx
+++ b/__docs/RoadMap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dev\exchange\RichLaughter3\__docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE92AF34-E7AD-49A6-A56E-8307045083E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6314DA61-1457-46BC-B4B6-508004CB3EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Тезисы" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="628">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1281" uniqueCount="638">
   <si>
     <t>RL3 - это продолжение RL1</t>
   </si>
@@ -1815,9 +1815,6 @@
     <t>Трейлинг-стоп по add_level</t>
   </si>
   <si>
-    <t>Узнать у разработчкиов cscalp, как мудрый поставил таймер на стаканы</t>
-  </si>
-  <si>
     <t>В тестер учет количество позитивных дней</t>
   </si>
   <si>
@@ -1951,6 +1948,39 @@
   </si>
   <si>
     <t>blender score</t>
+  </si>
+  <si>
+    <t>PEG17_AIUR</t>
+  </si>
+  <si>
+    <t>PEG17_PHOENIX попытка исправить текущие проблемы</t>
+  </si>
+  <si>
+    <t>PEG17_ALDERA</t>
+  </si>
+  <si>
+    <t>сестра PEG17_SELENDIS с использованием cvd</t>
+  </si>
+  <si>
+    <t>SID с отдельным скаченным датафреймом для истории</t>
+  </si>
+  <si>
+    <t>Сделать торговых роботов на perchan</t>
+  </si>
+  <si>
+    <t>Сделать торговых роботов на предолженных дипсиком индикаторах тренда</t>
+  </si>
+  <si>
+    <t>PEG26_JUNKRAT</t>
+  </si>
+  <si>
+    <t>PEG26_GAZLOWE</t>
+  </si>
+  <si>
+    <t>Модификация PEG26_UNKNOWN. Только контр-тренд</t>
+  </si>
+  <si>
+    <t>Модификация PEG26_UNKNOWN. С добавление пробоя</t>
   </si>
 </sst>
 </file>
@@ -2085,7 +2115,18 @@
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2407,95 +2448,95 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>605</v>
+      <c r="B2" t="s">
+        <v>573</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>606</v>
+      <c r="B3" t="s">
+        <v>588</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>607</v>
+      <c r="B4" t="s">
+        <v>591</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>608</v>
+      <c r="B5" t="s">
+        <v>599</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>609</v>
+      <c r="B6" t="s">
+        <v>602</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>610</v>
+      <c r="B7" t="s">
+        <v>620</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>627</v>
+      <c r="B8" t="s">
+        <v>597</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>616</v>
+      <c r="B9" t="s">
+        <v>598</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2503,32 +2544,32 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>621</v>
+      <c r="B11" s="17" t="s">
+        <v>632</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
-        <v>579</v>
+      <c r="B12" s="17" t="s">
+        <v>633</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2536,10 +2577,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2547,10 +2588,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2558,10 +2599,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -2569,10 +2610,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -2580,10 +2621,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="C17">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2591,10 +2632,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>612</v>
+        <v>566</v>
       </c>
       <c r="C18">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -2602,10 +2643,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>566</v>
+        <v>587</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -2613,10 +2654,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>582</v>
+        <v>622</v>
       </c>
       <c r="C20">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2624,10 +2665,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>598</v>
+        <v>592</v>
       </c>
       <c r="C21">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -2635,10 +2676,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -2646,10 +2687,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>600</v>
+        <v>589</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -2657,10 +2698,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -2668,10 +2709,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -2679,10 +2720,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>626</v>
+        <v>585</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -2690,10 +2731,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -2701,10 +2742,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>567</v>
+        <v>590</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -2712,10 +2753,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>568</v>
+        <v>583</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -2723,10 +2764,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>569</v>
+        <v>584</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2734,10 +2775,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -2745,10 +2786,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2756,10 +2797,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>572</v>
+        <v>616</v>
       </c>
       <c r="C33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -2767,10 +2808,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>573</v>
+        <v>619</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -2778,10 +2819,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -2789,10 +2830,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -2800,7 +2841,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>576</v>
+        <v>625</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -2811,7 +2852,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>577</v>
+        <v>593</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -2822,7 +2863,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>578</v>
+        <v>567</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -2833,7 +2874,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>584</v>
+        <v>569</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -2844,7 +2885,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>585</v>
+        <v>570</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2855,7 +2896,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>586</v>
+        <v>571</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -2866,7 +2907,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>587</v>
+        <v>572</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2877,7 +2918,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -2888,7 +2929,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2899,7 +2940,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2910,7 +2951,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>623</v>
+        <v>596</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -2921,7 +2962,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -2932,7 +2973,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>592</v>
+        <v>612</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -2943,7 +2984,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>593</v>
+        <v>613</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -2954,7 +2995,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>595</v>
+        <v>614</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2965,7 +3006,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>596</v>
+        <v>623</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2976,7 +3017,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>597</v>
+        <v>624</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -2986,8 +3027,8 @@
       <c r="A54">
         <v>53</v>
       </c>
-      <c r="B54" t="s">
-        <v>601</v>
+      <c r="B54" s="17" t="s">
+        <v>631</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -2997,99 +3038,111 @@
       <c r="A55">
         <v>54</v>
       </c>
-      <c r="B55" t="s">
-        <v>603</v>
+      <c r="B55" s="17" t="s">
+        <v>568</v>
       </c>
       <c r="C55">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
-      <c r="B56" t="s">
-        <v>613</v>
+      <c r="B56" s="17" t="s">
+        <v>574</v>
       </c>
       <c r="C56">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
-      <c r="B57" t="s">
-        <v>614</v>
+      <c r="B57" s="17" t="s">
+        <v>604</v>
       </c>
       <c r="C57">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
-      <c r="B58" t="s">
-        <v>615</v>
+      <c r="B58" s="17" t="s">
+        <v>605</v>
       </c>
       <c r="C58">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
-      <c r="B59" t="s">
-        <v>617</v>
+      <c r="B59" s="17" t="s">
+        <v>606</v>
       </c>
       <c r="C59">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
-      <c r="B60" t="s">
-        <v>620</v>
+      <c r="B60" s="17" t="s">
+        <v>607</v>
       </c>
       <c r="C60">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
-      <c r="B61" t="s">
-        <v>624</v>
+      <c r="B61" s="17" t="s">
+        <v>608</v>
       </c>
       <c r="C61">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
-      <c r="B62" t="s">
-        <v>625</v>
+      <c r="B62" s="17" t="s">
+        <v>609</v>
       </c>
       <c r="C62">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
+      <c r="B63" s="17" t="s">
+        <v>626</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
+      <c r="B64" s="17" t="s">
+        <v>615</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65">
@@ -4612,9 +4665,14 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C368">
-    <sortCondition descending="1" ref="C2:C368"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:C369">
+    <sortCondition descending="1" ref="C2:C369"/>
   </sortState>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7886,7 +7944,7 @@
       </c>
       <c r="L2">
         <f>COUNTIF(D:D,L1)</f>
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M2">
         <f>COUNTIF(D:D,M1)</f>
@@ -10530,20 +10588,68 @@
       <c r="A148">
         <v>147</v>
       </c>
+      <c r="B148" t="s">
+        <v>627</v>
+      </c>
+      <c r="C148" s="3">
+        <v>46318</v>
+      </c>
+      <c r="D148" t="s">
+        <v>12</v>
+      </c>
+      <c r="E148" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>148</v>
       </c>
+      <c r="B149" t="s">
+        <v>629</v>
+      </c>
+      <c r="C149" s="3">
+        <v>46318</v>
+      </c>
+      <c r="D149" t="s">
+        <v>12</v>
+      </c>
+      <c r="E149" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>149</v>
       </c>
+      <c r="B150" t="s">
+        <v>634</v>
+      </c>
+      <c r="C150" s="3">
+        <v>46318</v>
+      </c>
+      <c r="D150" t="s">
+        <v>12</v>
+      </c>
+      <c r="E150" t="s">
+        <v>636</v>
+      </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>635</v>
+      </c>
+      <c r="C151" s="3">
+        <v>46318</v>
+      </c>
+      <c r="D151" t="s">
+        <v>12</v>
+      </c>
+      <c r="E151" t="s">
+        <v>637</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>